<commit_message>
Phase 4-7: LSTM, PCA+MLP, advanced analysis, patient-specific model, IEEE report
- Phase 4: LSTM architecture (archived in src/archive/lstm/)
- Phase 5: PCA dimensionality reduction (242->25) + patient biometrics + compact MLP
- Phase 6: LOOCV, PCA scree plot, BW normalization, physics adherence, model comparison
- Phase 7: Patient-specific overfit model (Fz R2=0.884, RMSE=48N)
- Added 2D Clinical Dashboard (Dash/Plotly)
- IEEE-style report in report/IEEE_Report.md
</commit_message>
<xml_diff>
--- a/results/SimTK_Predictions.xlsx
+++ b/results/SimTK_Predictions.xlsx
@@ -443,13 +443,13 @@
         <v>1</v>
       </c>
       <c r="B2" t="n">
-        <v>178.0203717609386</v>
+        <v>265.7410374609464</v>
       </c>
       <c r="C2" t="n">
-        <v>-1487.058149733248</v>
+        <v>-1395.765062919586</v>
       </c>
       <c r="D2" t="n">
-        <v>1665.078521494187</v>
+        <v>1661.506100380532</v>
       </c>
     </row>
     <row r="3">
@@ -457,13 +457,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>185.2872323738582</v>
+        <v>256.1273995400389</v>
       </c>
       <c r="C3" t="n">
-        <v>-1476.517096768002</v>
+        <v>-1396.664163410899</v>
       </c>
       <c r="D3" t="n">
-        <v>1661.804329141861</v>
+        <v>1652.791562950938</v>
       </c>
     </row>
     <row r="4">
@@ -471,13 +471,13 @@
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>202.1081722665314</v>
+        <v>261.7878557393394</v>
       </c>
       <c r="C4" t="n">
-        <v>-1463.647458612875</v>
+        <v>-1394.640665379309</v>
       </c>
       <c r="D4" t="n">
-        <v>1665.755630879407</v>
+        <v>1656.428521118648</v>
       </c>
     </row>
     <row r="5">
@@ -485,13 +485,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="n">
-        <v>172.0137889238068</v>
+        <v>261.9738606962721</v>
       </c>
       <c r="C5" t="n">
-        <v>-1485.963781278191</v>
+        <v>-1392.478652830632</v>
       </c>
       <c r="D5" t="n">
-        <v>1657.977570201998</v>
+        <v>1654.452513526905</v>
       </c>
     </row>
     <row r="6">
@@ -499,13 +499,13 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>182.4300628614476</v>
+        <v>265.7148349250496</v>
       </c>
       <c r="C6" t="n">
-        <v>-1481.344344418595</v>
+        <v>-1389.120849018293</v>
       </c>
       <c r="D6" t="n">
-        <v>1663.774407280042</v>
+        <v>1654.835683943343</v>
       </c>
     </row>
     <row r="7">
@@ -513,13 +513,13 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>182.1810884848093</v>
+        <v>273.7857233769681</v>
       </c>
       <c r="C7" t="n">
-        <v>-1475.506597346421</v>
+        <v>-1384.806255420177</v>
       </c>
       <c r="D7" t="n">
-        <v>1657.68768583123</v>
+        <v>1658.591978797145</v>
       </c>
     </row>
     <row r="8">
@@ -527,13 +527,13 @@
         <v>7</v>
       </c>
       <c r="B8" t="n">
-        <v>178.1457278985525</v>
+        <v>276.7773587653306</v>
       </c>
       <c r="C8" t="n">
-        <v>-1501.198502601014</v>
+        <v>-1380.415576492917</v>
       </c>
       <c r="D8" t="n">
-        <v>1679.344230499567</v>
+        <v>1657.192935258247</v>
       </c>
     </row>
     <row r="9">
@@ -541,13 +541,13 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>183.6472537581708</v>
+        <v>299.6758064514928</v>
       </c>
       <c r="C9" t="n">
-        <v>-1502.394741275538</v>
+        <v>-1368.713186446162</v>
       </c>
       <c r="D9" t="n">
-        <v>1686.041995033709</v>
+        <v>1668.388992897655</v>
       </c>
     </row>
     <row r="10">
@@ -555,13 +555,13 @@
         <v>9</v>
       </c>
       <c r="B10" t="n">
-        <v>187.4958380693527</v>
+        <v>283.2845287329831</v>
       </c>
       <c r="C10" t="n">
-        <v>-1504.553900305762</v>
+        <v>-1376.159636527828</v>
       </c>
       <c r="D10" t="n">
-        <v>1692.049738375115</v>
+        <v>1659.444165260812</v>
       </c>
     </row>
     <row r="11">
@@ -569,13 +569,13 @@
         <v>10</v>
       </c>
       <c r="B11" t="n">
-        <v>190.8754248035687</v>
+        <v>279.6521066513831</v>
       </c>
       <c r="C11" t="n">
-        <v>-1480.920624819159</v>
+        <v>-1380.158087109908</v>
       </c>
       <c r="D11" t="n">
-        <v>1671.796049622728</v>
+        <v>1659.810193761291</v>
       </c>
     </row>
     <row r="12">
@@ -583,13 +583,13 @@
         <v>11</v>
       </c>
       <c r="B12" t="n">
-        <v>182.1243609485074</v>
+        <v>282.5483069408138</v>
       </c>
       <c r="C12" t="n">
-        <v>-1495.074131371231</v>
+        <v>-1378.784083341904</v>
       </c>
       <c r="D12" t="n">
-        <v>1677.198492319738</v>
+        <v>1661.332390282717</v>
       </c>
     </row>
     <row r="13">
@@ -597,13 +597,13 @@
         <v>12</v>
       </c>
       <c r="B13" t="n">
-        <v>174.6024438088799</v>
+        <v>275.5154092609657</v>
       </c>
       <c r="C13" t="n">
-        <v>-1485.161815897559</v>
+        <v>-1382.359320114497</v>
       </c>
       <c r="D13" t="n">
-        <v>1659.764259706439</v>
+        <v>1657.874729375462</v>
       </c>
     </row>
     <row r="14">
@@ -611,13 +611,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="n">
-        <v>171.4324597316009</v>
+        <v>278.5920185338418</v>
       </c>
       <c r="C14" t="n">
-        <v>-1483.880107596545</v>
+        <v>-1381.353049648332</v>
       </c>
       <c r="D14" t="n">
-        <v>1655.312567328146</v>
+        <v>1659.945068182173</v>
       </c>
     </row>
     <row r="15">
@@ -625,13 +625,13 @@
         <v>14</v>
       </c>
       <c r="B15" t="n">
-        <v>174.5282378935859</v>
+        <v>261.083219852066</v>
       </c>
       <c r="C15" t="n">
-        <v>-1467.598491762494</v>
+        <v>-1390.872380647365</v>
       </c>
       <c r="D15" t="n">
-        <v>1642.12672965608</v>
+        <v>1651.955600499431</v>
       </c>
     </row>
     <row r="16">
@@ -639,13 +639,13 @@
         <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>171.0515921936952</v>
+        <v>247.5885109434636</v>
       </c>
       <c r="C16" t="n">
-        <v>-1457.585076476637</v>
+        <v>-1397.965404617132</v>
       </c>
       <c r="D16" t="n">
-        <v>1628.636668670333</v>
+        <v>1645.553915560595</v>
       </c>
     </row>
     <row r="17">
@@ -653,13 +653,13 @@
         <v>16</v>
       </c>
       <c r="B17" t="n">
-        <v>171.1056416778623</v>
+        <v>245.4427822546913</v>
       </c>
       <c r="C17" t="n">
-        <v>-1454.909776694405</v>
+        <v>-1399.487487207312</v>
       </c>
       <c r="D17" t="n">
-        <v>1626.015418372267</v>
+        <v>1644.930269462003</v>
       </c>
     </row>
     <row r="18">
@@ -667,13 +667,13 @@
         <v>17</v>
       </c>
       <c r="B18" t="n">
-        <v>171.4232528069206</v>
+        <v>242.1028556339978</v>
       </c>
       <c r="C18" t="n">
-        <v>-1454.182131529902</v>
+        <v>-1400.329586418139</v>
       </c>
       <c r="D18" t="n">
-        <v>1625.605384336823</v>
+        <v>1642.432442052137</v>
       </c>
     </row>
     <row r="19">
@@ -681,13 +681,13 @@
         <v>18</v>
       </c>
       <c r="B19" t="n">
-        <v>170.4342126852906</v>
+        <v>241.8915958016489</v>
       </c>
       <c r="C19" t="n">
-        <v>-1458.425016782393</v>
+        <v>-1400.097235188214</v>
       </c>
       <c r="D19" t="n">
-        <v>1628.859229467684</v>
+        <v>1641.988830989863</v>
       </c>
     </row>
     <row r="20">
@@ -695,13 +695,13 @@
         <v>19</v>
       </c>
       <c r="B20" t="n">
-        <v>167.1055359213587</v>
+        <v>241.3322236825495</v>
       </c>
       <c r="C20" t="n">
-        <v>-1460.909577457358</v>
+        <v>-1400.508119267251</v>
       </c>
       <c r="D20" t="n">
-        <v>1628.015113378717</v>
+        <v>1641.8403429498</v>
       </c>
     </row>
     <row r="21">
@@ -709,13 +709,13 @@
         <v>20</v>
       </c>
       <c r="B21" t="n">
-        <v>167.3980261578714</v>
+        <v>239.1379885409572</v>
       </c>
       <c r="C21" t="n">
-        <v>-1466.82962234395</v>
+        <v>-1402.331641942453</v>
       </c>
       <c r="D21" t="n">
-        <v>1634.227648501821</v>
+        <v>1641.46963048341</v>
       </c>
     </row>
     <row r="22">
@@ -723,13 +723,13 @@
         <v>21</v>
       </c>
       <c r="B22" t="n">
-        <v>162.9363633188181</v>
+        <v>236.2726611508998</v>
       </c>
       <c r="C22" t="n">
-        <v>-1475.330648361616</v>
+        <v>-1403.772127384827</v>
       </c>
       <c r="D22" t="n">
-        <v>1638.267011680434</v>
+        <v>1640.044788535726</v>
       </c>
     </row>
     <row r="23">
@@ -737,13 +737,13 @@
         <v>22</v>
       </c>
       <c r="B23" t="n">
-        <v>155.3843683741386</v>
+        <v>230.9924303065527</v>
       </c>
       <c r="C23" t="n">
-        <v>-1486.133963129256</v>
+        <v>-1407.784851759317</v>
       </c>
       <c r="D23" t="n">
-        <v>1641.518331503394</v>
+        <v>1638.77728206587</v>
       </c>
     </row>
     <row r="24">
@@ -751,13 +751,13 @@
         <v>23</v>
       </c>
       <c r="B24" t="n">
-        <v>161.2087582466354</v>
+        <v>228.5970680516126</v>
       </c>
       <c r="C24" t="n">
-        <v>-1484.932441078868</v>
+        <v>-1409.123392204682</v>
       </c>
       <c r="D24" t="n">
-        <v>1646.141199325504</v>
+        <v>1637.720460256295</v>
       </c>
     </row>
     <row r="25">
@@ -765,13 +765,13 @@
         <v>24</v>
       </c>
       <c r="B25" t="n">
-        <v>157.4046343398926</v>
+        <v>229.9161908739013</v>
       </c>
       <c r="C25" t="n">
-        <v>-1488.720122661077</v>
+        <v>-1408.551594743946</v>
       </c>
       <c r="D25" t="n">
-        <v>1646.124757000969</v>
+        <v>1638.467785617847</v>
       </c>
     </row>
     <row r="26">
@@ -779,13 +779,13 @@
         <v>25</v>
       </c>
       <c r="B26" t="n">
-        <v>167.1584358733151</v>
+        <v>231.27744593327</v>
       </c>
       <c r="C26" t="n">
-        <v>-1481.583480005191</v>
+        <v>-1407.89085786486</v>
       </c>
       <c r="D26" t="n">
-        <v>1648.741915878506</v>
+        <v>1639.16830379813</v>
       </c>
     </row>
     <row r="27">
@@ -793,13 +793,13 @@
         <v>26</v>
       </c>
       <c r="B27" t="n">
-        <v>151.1964038050518</v>
+        <v>236.3680116832406</v>
       </c>
       <c r="C27" t="n">
-        <v>-1487.039771372172</v>
+        <v>-1405.736900873176</v>
       </c>
       <c r="D27" t="n">
-        <v>1638.236175177224</v>
+        <v>1642.104912556417</v>
       </c>
     </row>
     <row r="28">
@@ -807,13 +807,13 @@
         <v>27</v>
       </c>
       <c r="B28" t="n">
-        <v>168.3370654563404</v>
+        <v>242.7652502119232</v>
       </c>
       <c r="C28" t="n">
-        <v>-1472.13567466872</v>
+        <v>-1404.460102023835</v>
       </c>
       <c r="D28" t="n">
-        <v>1640.47274012506</v>
+        <v>1647.225352235758</v>
       </c>
     </row>
     <row r="29">
@@ -821,13 +821,13 @@
         <v>28</v>
       </c>
       <c r="B29" t="n">
-        <v>151.7017802039178</v>
+        <v>251.289641678357</v>
       </c>
       <c r="C29" t="n">
-        <v>-1474.052106155035</v>
+        <v>-1401.757376529935</v>
       </c>
       <c r="D29" t="n">
-        <v>1625.753886358953</v>
+        <v>1653.047018208292</v>
       </c>
     </row>
     <row r="30">
@@ -835,13 +835,13 @@
         <v>29</v>
       </c>
       <c r="B30" t="n">
-        <v>166.3004122387624</v>
+        <v>241.771773122082</v>
       </c>
       <c r="C30" t="n">
-        <v>-1469.7413657129</v>
+        <v>-1404.02263823907</v>
       </c>
       <c r="D30" t="n">
-        <v>1636.041777951663</v>
+        <v>1645.794411361152</v>
       </c>
     </row>
     <row r="31">
@@ -849,13 +849,13 @@
         <v>30</v>
       </c>
       <c r="B31" t="n">
-        <v>170.8984412969314</v>
+        <v>236.8883556702825</v>
       </c>
       <c r="C31" t="n">
-        <v>-1468.384872596336</v>
+        <v>-1405.833688155661</v>
       </c>
       <c r="D31" t="n">
-        <v>1639.283313893267</v>
+        <v>1642.722043825943</v>
       </c>
     </row>
     <row r="32">
@@ -863,13 +863,13 @@
         <v>31</v>
       </c>
       <c r="B32" t="n">
-        <v>165.6948663617119</v>
+        <v>238.5271776016091</v>
       </c>
       <c r="C32" t="n">
-        <v>-1463.480109499246</v>
+        <v>-1406.147652483285</v>
       </c>
       <c r="D32" t="n">
-        <v>1629.174975860958</v>
+        <v>1644.674830084894</v>
       </c>
     </row>
     <row r="33">
@@ -877,13 +877,13 @@
         <v>32</v>
       </c>
       <c r="B33" t="n">
-        <v>164.0762604529984</v>
+        <v>231.8426595772788</v>
       </c>
       <c r="C33" t="n">
-        <v>-1464.704278347133</v>
+        <v>-1409.744742742246</v>
       </c>
       <c r="D33" t="n">
-        <v>1628.780538800132</v>
+        <v>1641.587402319524</v>
       </c>
     </row>
     <row r="34">
@@ -891,13 +891,13 @@
         <v>33</v>
       </c>
       <c r="B34" t="n">
-        <v>156.3121866926386</v>
+        <v>232.1923700567604</v>
       </c>
       <c r="C34" t="n">
-        <v>-1463.796936439464</v>
+        <v>-1411.216353092834</v>
       </c>
       <c r="D34" t="n">
-        <v>1620.109123132103</v>
+        <v>1643.408723149594</v>
       </c>
     </row>
     <row r="35">
@@ -905,13 +905,13 @@
         <v>34</v>
       </c>
       <c r="B35" t="n">
-        <v>156.5143227110328</v>
+        <v>219.9095783583233</v>
       </c>
       <c r="C35" t="n">
-        <v>-1469.605043040709</v>
+        <v>-1417.754605667163</v>
       </c>
       <c r="D35" t="n">
-        <v>1626.119365751742</v>
+        <v>1637.664184025487</v>
       </c>
     </row>
     <row r="36">
@@ -919,13 +919,13 @@
         <v>35</v>
       </c>
       <c r="B36" t="n">
-        <v>158.7470034465129</v>
+        <v>214.3558012315661</v>
       </c>
       <c r="C36" t="n">
-        <v>-1475.357896623946</v>
+        <v>-1421.590394829965</v>
       </c>
       <c r="D36" t="n">
-        <v>1634.104900070459</v>
+        <v>1635.946196061531</v>
       </c>
     </row>
     <row r="37">
@@ -933,13 +933,13 @@
         <v>36</v>
       </c>
       <c r="B37" t="n">
-        <v>158.961337586792</v>
+        <v>210.4774776014645</v>
       </c>
       <c r="C37" t="n">
-        <v>-1479.502422868804</v>
+        <v>-1424.600469727975</v>
       </c>
       <c r="D37" t="n">
-        <v>1638.463760455596</v>
+        <v>1635.07794732944</v>
       </c>
     </row>
     <row r="38">
@@ -947,13 +947,13 @@
         <v>37</v>
       </c>
       <c r="B38" t="n">
-        <v>168.0149013385073</v>
+        <v>215.6390660251869</v>
       </c>
       <c r="C38" t="n">
-        <v>-1487.647765621881</v>
+        <v>-1425.275687192811</v>
       </c>
       <c r="D38" t="n">
-        <v>1655.662666960388</v>
+        <v>1640.914753217997</v>
       </c>
     </row>
     <row r="39">
@@ -961,13 +961,13 @@
         <v>38</v>
       </c>
       <c r="B39" t="n">
-        <v>151.7081438113354</v>
+        <v>207.8311376313379</v>
       </c>
       <c r="C39" t="n">
-        <v>-1489.857146628121</v>
+        <v>-1429.012841733821</v>
       </c>
       <c r="D39" t="n">
-        <v>1641.565290439457</v>
+        <v>1636.84397936516</v>
       </c>
     </row>
     <row r="40">
@@ -975,13 +975,13 @@
         <v>39</v>
       </c>
       <c r="B40" t="n">
-        <v>178.3239630003274</v>
+        <v>205.594453306205</v>
       </c>
       <c r="C40" t="n">
-        <v>-1484.943472465639</v>
+        <v>-1432.804055185896</v>
       </c>
       <c r="D40" t="n">
-        <v>1663.267435465966</v>
+        <v>1638.398508492101</v>
       </c>
     </row>
     <row r="41">
@@ -989,13 +989,13 @@
         <v>40</v>
       </c>
       <c r="B41" t="n">
-        <v>143.484885252692</v>
+        <v>200.1003369561396</v>
       </c>
       <c r="C41" t="n">
-        <v>-1491.338617340619</v>
+        <v>-1435.084165077016</v>
       </c>
       <c r="D41" t="n">
-        <v>1634.823502593311</v>
+        <v>1635.184502033156</v>
       </c>
     </row>
     <row r="42">
@@ -1003,13 +1003,13 @@
         <v>41</v>
       </c>
       <c r="B42" t="n">
-        <v>234.8676074061798</v>
+        <v>248.1566395003039</v>
       </c>
       <c r="C42" t="n">
-        <v>-1422.481218718115</v>
+        <v>-1423.415760850221</v>
       </c>
       <c r="D42" t="n">
-        <v>1657.348826124295</v>
+        <v>1671.572400350525</v>
       </c>
     </row>
     <row r="43">
@@ -1017,13 +1017,13 @@
         <v>42</v>
       </c>
       <c r="B43" t="n">
-        <v>267.2746434451588</v>
+        <v>255.22219253552</v>
       </c>
       <c r="C43" t="n">
-        <v>-1403.736327236724</v>
+        <v>-1430.42478146042</v>
       </c>
       <c r="D43" t="n">
-        <v>1671.010970681883</v>
+        <v>1685.646973995939</v>
       </c>
     </row>
     <row r="44">
@@ -1031,13 +1031,13 @@
         <v>43</v>
       </c>
       <c r="B44" t="n">
-        <v>258.0604308475308</v>
+        <v>233.3812360152909</v>
       </c>
       <c r="C44" t="n">
-        <v>-1421.061293187419</v>
+        <v>-1433.422592437979</v>
       </c>
       <c r="D44" t="n">
-        <v>1679.12172403495</v>
+        <v>1666.80382845327</v>
       </c>
     </row>
     <row r="45">
@@ -1045,13 +1045,13 @@
         <v>44</v>
       </c>
       <c r="B45" t="n">
-        <v>233.9060630115615</v>
+        <v>224.9253268571261</v>
       </c>
       <c r="C45" t="n">
-        <v>-1491.088711555787</v>
+        <v>-1415.009105505442</v>
       </c>
       <c r="D45" t="n">
-        <v>1724.994774567348</v>
+        <v>1639.934432362568</v>
       </c>
     </row>
     <row r="46">
@@ -1059,13 +1059,13 @@
         <v>45</v>
       </c>
       <c r="B46" t="n">
-        <v>175.9255094092905</v>
+        <v>239.2654683749856</v>
       </c>
       <c r="C46" t="n">
-        <v>-1471.839933219933</v>
+        <v>-1392.638558405856</v>
       </c>
       <c r="D46" t="n">
-        <v>1647.765442629224</v>
+        <v>1631.904026780841</v>
       </c>
     </row>
     <row r="47">
@@ -1073,13 +1073,13 @@
         <v>46</v>
       </c>
       <c r="B47" t="n">
-        <v>182.6767287714907</v>
+        <v>273.1696554760642</v>
       </c>
       <c r="C47" t="n">
-        <v>-1454.534086033738</v>
+        <v>-1380.263708296657</v>
       </c>
       <c r="D47" t="n">
-        <v>1637.210814805229</v>
+        <v>1653.433363772722</v>
       </c>
     </row>
     <row r="48">
@@ -1087,13 +1087,13 @@
         <v>47</v>
       </c>
       <c r="B48" t="n">
-        <v>176.0093214988143</v>
+        <v>256.7585623404499</v>
       </c>
       <c r="C48" t="n">
-        <v>-1445.302963063603</v>
+        <v>-1386.939944701951</v>
       </c>
       <c r="D48" t="n">
-        <v>1621.312284562418</v>
+        <v>1643.6985070424</v>
       </c>
     </row>
     <row r="49">
@@ -1101,13 +1101,13 @@
         <v>48</v>
       </c>
       <c r="B49" t="n">
-        <v>186.3976049028944</v>
+        <v>246.9703447612133</v>
       </c>
       <c r="C49" t="n">
-        <v>-1449.680039051641</v>
+        <v>-1395.927938654158</v>
       </c>
       <c r="D49" t="n">
-        <v>1636.077643954535</v>
+        <v>1642.898283415371</v>
       </c>
     </row>
     <row r="50">
@@ -1115,13 +1115,13 @@
         <v>49</v>
       </c>
       <c r="B50" t="n">
-        <v>179.8768577460567</v>
+        <v>275.4900277872671</v>
       </c>
       <c r="C50" t="n">
-        <v>-1438.690957283975</v>
+        <v>-1382.74261104392</v>
       </c>
       <c r="D50" t="n">
-        <v>1618.567815030032</v>
+        <v>1658.232638831187</v>
       </c>
     </row>
     <row r="51">
@@ -1129,13 +1129,13 @@
         <v>50</v>
       </c>
       <c r="B51" t="n">
-        <v>187.3317991264794</v>
+        <v>252.3867283796386</v>
       </c>
       <c r="C51" t="n">
-        <v>-1451.889608400233</v>
+        <v>-1395.177170340826</v>
       </c>
       <c r="D51" t="n">
-        <v>1639.221407526712</v>
+        <v>1647.563898720465</v>
       </c>
     </row>
     <row r="52">
@@ -1143,13 +1143,13 @@
         <v>51</v>
       </c>
       <c r="B52" t="n">
-        <v>166.0334345640462</v>
+        <v>263.2583237883584</v>
       </c>
       <c r="C52" t="n">
-        <v>-1439.281203778057</v>
+        <v>-1391.616145354416</v>
       </c>
       <c r="D52" t="n">
-        <v>1605.314638342104</v>
+        <v>1654.874469142774</v>
       </c>
     </row>
     <row r="53">
@@ -1157,13 +1157,13 @@
         <v>52</v>
       </c>
       <c r="B53" t="n">
-        <v>185.2576371085783</v>
+        <v>265.0824193637793</v>
       </c>
       <c r="C53" t="n">
-        <v>-1430.583551692548</v>
+        <v>-1395.678738758588</v>
       </c>
       <c r="D53" t="n">
-        <v>1615.841188801127</v>
+        <v>1660.761158122367</v>
       </c>
     </row>
     <row r="54">
@@ -1171,13 +1171,13 @@
         <v>53</v>
       </c>
       <c r="B54" t="n">
-        <v>183.9201794310869</v>
+        <v>263.580406263952</v>
       </c>
       <c r="C54" t="n">
-        <v>-1444.497303496346</v>
+        <v>-1397.306224873863</v>
       </c>
       <c r="D54" t="n">
-        <v>1628.417482927433</v>
+        <v>1660.886631137815</v>
       </c>
     </row>
     <row r="55">
@@ -1185,13 +1185,13 @@
         <v>54</v>
       </c>
       <c r="B55" t="n">
-        <v>179.7679925619695</v>
+        <v>282.6081763770715</v>
       </c>
       <c r="C55" t="n">
-        <v>-1422.87167029781</v>
+        <v>-1383.226915533704</v>
       </c>
       <c r="D55" t="n">
-        <v>1602.63966285978</v>
+        <v>1665.835091910776</v>
       </c>
     </row>
     <row r="56">
@@ -1199,13 +1199,13 @@
         <v>55</v>
       </c>
       <c r="B56" t="n">
-        <v>186.0394162834309</v>
+        <v>279.7160338391157</v>
       </c>
       <c r="C56" t="n">
-        <v>-1413.230066614493</v>
+        <v>-1386.388122381127</v>
       </c>
       <c r="D56" t="n">
-        <v>1599.269482897924</v>
+        <v>1666.104156220243</v>
       </c>
     </row>
     <row r="57">
@@ -1213,13 +1213,13 @@
         <v>56</v>
       </c>
       <c r="B57" t="n">
-        <v>178.3038260270069</v>
+        <v>269.4920252132965</v>
       </c>
       <c r="C57" t="n">
-        <v>-1430.152567277769</v>
+        <v>-1390.30321292485</v>
       </c>
       <c r="D57" t="n">
-        <v>1608.456393304776</v>
+        <v>1659.795238138147</v>
       </c>
     </row>
     <row r="58">
@@ -1227,13 +1227,13 @@
         <v>57</v>
       </c>
       <c r="B58" t="n">
-        <v>173.2005826719597</v>
+        <v>261.9555784423341</v>
       </c>
       <c r="C58" t="n">
-        <v>-1430.149345689538</v>
+        <v>-1393.595445075439</v>
       </c>
       <c r="D58" t="n">
-        <v>1603.349928361498</v>
+        <v>1655.551023517773</v>
       </c>
     </row>
     <row r="59">
@@ -1241,13 +1241,13 @@
         <v>58</v>
       </c>
       <c r="B59" t="n">
-        <v>176.0951858105623</v>
+        <v>261.0446033115903</v>
       </c>
       <c r="C59" t="n">
-        <v>-1426.567345854415</v>
+        <v>-1393.038466038949</v>
       </c>
       <c r="D59" t="n">
-        <v>1602.662531664977</v>
+        <v>1654.08306935054</v>
       </c>
     </row>
     <row r="60">
@@ -1255,13 +1255,13 @@
         <v>59</v>
       </c>
       <c r="B60" t="n">
-        <v>161.5653569531565</v>
+        <v>262.540601262844</v>
       </c>
       <c r="C60" t="n">
-        <v>-1438.803678225916</v>
+        <v>-1391.545465400984</v>
       </c>
       <c r="D60" t="n">
-        <v>1600.369035179072</v>
+        <v>1654.086066663828</v>
       </c>
     </row>
     <row r="61">
@@ -1269,13 +1269,13 @@
         <v>60</v>
       </c>
       <c r="B61" t="n">
-        <v>173.9891231547347</v>
+        <v>256.9789326944663</v>
       </c>
       <c r="C61" t="n">
-        <v>-1427.919508434537</v>
+        <v>-1392.410713866015</v>
       </c>
       <c r="D61" t="n">
-        <v>1601.908631589271</v>
+        <v>1649.389646560481</v>
       </c>
     </row>
     <row r="62">
@@ -1283,13 +1283,13 @@
         <v>61</v>
       </c>
       <c r="B62" t="n">
-        <v>163.7750778508151</v>
+        <v>264.2936772841204</v>
       </c>
       <c r="C62" t="n">
-        <v>-1430.899610751551</v>
+        <v>-1387.477638428032</v>
       </c>
       <c r="D62" t="n">
-        <v>1594.674688602367</v>
+        <v>1651.771315712153</v>
       </c>
     </row>
     <row r="63">
@@ -1297,13 +1297,13 @@
         <v>62</v>
       </c>
       <c r="B63" t="n">
-        <v>163.0615783925191</v>
+        <v>261.651789227595</v>
       </c>
       <c r="C63" t="n">
-        <v>-1432.950435595067</v>
+        <v>-1387.123730641547</v>
       </c>
       <c r="D63" t="n">
-        <v>1596.012013987586</v>
+        <v>1648.775519869142</v>
       </c>
     </row>
     <row r="64">
@@ -1311,13 +1311,13 @@
         <v>63</v>
       </c>
       <c r="B64" t="n">
-        <v>142.9539054357621</v>
+        <v>255.0846759711539</v>
       </c>
       <c r="C64" t="n">
-        <v>-1450.895629662718</v>
+        <v>-1387.553146688142</v>
       </c>
       <c r="D64" t="n">
-        <v>1593.84953509848</v>
+        <v>1642.637822659296</v>
       </c>
     </row>
     <row r="65">
@@ -1325,13 +1325,13 @@
         <v>64</v>
       </c>
       <c r="B65" t="n">
-        <v>151.5404731424896</v>
+        <v>261.2422957328067</v>
       </c>
       <c r="C65" t="n">
-        <v>-1445.105174110775</v>
+        <v>-1380.69319881539</v>
       </c>
       <c r="D65" t="n">
-        <v>1596.645647253265</v>
+        <v>1641.935494548197</v>
       </c>
     </row>
     <row r="66">
@@ -1339,13 +1339,13 @@
         <v>65</v>
       </c>
       <c r="B66" t="n">
-        <v>149.2577389668234</v>
+        <v>289.540385104358</v>
       </c>
       <c r="C66" t="n">
-        <v>-1443.946025446035</v>
+        <v>-1368.383322768365</v>
       </c>
       <c r="D66" t="n">
-        <v>1593.203764412858</v>
+        <v>1657.923707872723</v>
       </c>
     </row>
     <row r="67">
@@ -1353,13 +1353,13 @@
         <v>66</v>
       </c>
       <c r="B67" t="n">
-        <v>154.2574039102024</v>
+        <v>302.199055462352</v>
       </c>
       <c r="C67" t="n">
-        <v>-1438.59681784546</v>
+        <v>-1363.952377078832</v>
       </c>
       <c r="D67" t="n">
-        <v>1592.854221755662</v>
+        <v>1666.151432541184</v>
       </c>
     </row>
     <row r="68">
@@ -1367,13 +1367,13 @@
         <v>67</v>
       </c>
       <c r="B68" t="n">
-        <v>154.4994327527371</v>
+        <v>310.960978651265</v>
       </c>
       <c r="C68" t="n">
-        <v>-1437.378203899937</v>
+        <v>-1360.48823572992</v>
       </c>
       <c r="D68" t="n">
-        <v>1591.877636652674</v>
+        <v>1671.449214381186</v>
       </c>
     </row>
     <row r="69">
@@ -1381,13 +1381,13 @@
         <v>68</v>
       </c>
       <c r="B69" t="n">
-        <v>151.4443825121115</v>
+        <v>312.2348945250085</v>
       </c>
       <c r="C69" t="n">
-        <v>-1437.389073222863</v>
+        <v>-1362.114850781484</v>
       </c>
       <c r="D69" t="n">
-        <v>1588.833455734975</v>
+        <v>1674.349745306493</v>
       </c>
     </row>
     <row r="70">
@@ -1395,13 +1395,13 @@
         <v>69</v>
       </c>
       <c r="B70" t="n">
-        <v>143.0806678214151</v>
+        <v>317.2230855455197</v>
       </c>
       <c r="C70" t="n">
-        <v>-1441.550450359917</v>
+        <v>-1357.229120693137</v>
       </c>
       <c r="D70" t="n">
-        <v>1584.631118181332</v>
+        <v>1674.452206238656</v>
       </c>
     </row>
     <row r="71">
@@ -1409,13 +1409,13 @@
         <v>70</v>
       </c>
       <c r="B71" t="n">
-        <v>74.32216523572924</v>
+        <v>220.4159582434116</v>
       </c>
       <c r="C71" t="n">
-        <v>-1475.9481457697</v>
+        <v>-1420.92817522368</v>
       </c>
       <c r="D71" t="n">
-        <v>1550.270311005429</v>
+        <v>1641.344133467092</v>
       </c>
     </row>
     <row r="72">
@@ -1423,13 +1423,13 @@
         <v>71</v>
       </c>
       <c r="B72" t="n">
-        <v>76.00740987162962</v>
+        <v>227.7536073472756</v>
       </c>
       <c r="C72" t="n">
-        <v>-1501.474574861474</v>
+        <v>-1407.658151865425</v>
       </c>
       <c r="D72" t="n">
-        <v>1577.481984733104</v>
+        <v>1635.4117592127</v>
       </c>
     </row>
     <row r="73">
@@ -1437,13 +1437,13 @@
         <v>72</v>
       </c>
       <c r="B73" t="n">
-        <v>87.60854419628815</v>
+        <v>232.9593268898113</v>
       </c>
       <c r="C73" t="n">
-        <v>-1494.309571000204</v>
+        <v>-1397.063878953393</v>
       </c>
       <c r="D73" t="n">
-        <v>1581.918115196492</v>
+        <v>1630.023205843204</v>
       </c>
     </row>
     <row r="74">
@@ -1451,13 +1451,13 @@
         <v>73</v>
       </c>
       <c r="B74" t="n">
-        <v>107.2722925711817</v>
+        <v>232.1528202215631</v>
       </c>
       <c r="C74" t="n">
-        <v>-1486.481255150449</v>
+        <v>-1393.850492549107</v>
       </c>
       <c r="D74" t="n">
-        <v>1593.753547721631</v>
+        <v>1626.003312770671</v>
       </c>
     </row>
     <row r="75">
@@ -1465,13 +1465,13 @@
         <v>74</v>
       </c>
       <c r="B75" t="n">
-        <v>108.1467860580034</v>
+        <v>207.2266694222105</v>
       </c>
       <c r="C75" t="n">
-        <v>-1479.83109041215</v>
+        <v>-1405.64907505722</v>
       </c>
       <c r="D75" t="n">
-        <v>1587.977876470154</v>
+        <v>1612.875744479431</v>
       </c>
     </row>
     <row r="76">
@@ -1479,13 +1479,13 @@
         <v>75</v>
       </c>
       <c r="B76" t="n">
-        <v>109.1768928801044</v>
+        <v>194.1846558518602</v>
       </c>
       <c r="C76" t="n">
-        <v>-1477.735374428417</v>
+        <v>-1394.984564448255</v>
       </c>
       <c r="D76" t="n">
-        <v>1586.912267308522</v>
+        <v>1589.169220300115</v>
       </c>
     </row>
     <row r="77">
@@ -1493,13 +1493,13 @@
         <v>76</v>
       </c>
       <c r="B77" t="n">
-        <v>108.2478249180338</v>
+        <v>177.2800152218248</v>
       </c>
       <c r="C77" t="n">
-        <v>-1483.23184830765</v>
+        <v>-1404.983976415542</v>
       </c>
       <c r="D77" t="n">
-        <v>1591.479673225684</v>
+        <v>1582.263991637366</v>
       </c>
     </row>
     <row r="78">
@@ -1507,13 +1507,13 @@
         <v>77</v>
       </c>
       <c r="B78" t="n">
-        <v>97.96674216990139</v>
+        <v>161.9946248353264</v>
       </c>
       <c r="C78" t="n">
-        <v>-1500.017848849376</v>
+        <v>-1419.630948218389</v>
       </c>
       <c r="D78" t="n">
-        <v>1597.984591019277</v>
+        <v>1581.625573053715</v>
       </c>
     </row>
     <row r="79">
@@ -1521,13 +1521,13 @@
         <v>78</v>
       </c>
       <c r="B79" t="n">
-        <v>112.1375813431588</v>
+        <v>155.2121910003362</v>
       </c>
       <c r="C79" t="n">
-        <v>-1484.297179049176</v>
+        <v>-1426.824422666585</v>
       </c>
       <c r="D79" t="n">
-        <v>1596.434760392335</v>
+        <v>1582.036613666921</v>
       </c>
     </row>
     <row r="80">
@@ -1535,13 +1535,13 @@
         <v>79</v>
       </c>
       <c r="B80" t="n">
-        <v>149.0351692011689</v>
+        <v>141.9072786995002</v>
       </c>
       <c r="C80" t="n">
-        <v>-1454.368318755159</v>
+        <v>-1429.595631331829</v>
       </c>
       <c r="D80" t="n">
-        <v>1603.403487956328</v>
+        <v>1571.502910031329</v>
       </c>
     </row>
     <row r="81">
@@ -1549,13 +1549,13 @@
         <v>80</v>
       </c>
       <c r="B81" t="n">
-        <v>158.9676801184137</v>
+        <v>105.0120852193399</v>
       </c>
       <c r="C81" t="n">
-        <v>-1449.938624896569</v>
+        <v>-1454.863263878754</v>
       </c>
       <c r="D81" t="n">
-        <v>1608.906305014983</v>
+        <v>1559.875349098094</v>
       </c>
     </row>
     <row r="82">
@@ -1563,13 +1563,13 @@
         <v>81</v>
       </c>
       <c r="B82" t="n">
-        <v>160.7055657704563</v>
+        <v>100.5199728213107</v>
       </c>
       <c r="C82" t="n">
-        <v>-1450.196170198442</v>
+        <v>-1459.084116506499</v>
       </c>
       <c r="D82" t="n">
-        <v>1610.901735968898</v>
+        <v>1559.60408932781</v>
       </c>
     </row>
     <row r="83">
@@ -1577,13 +1577,13 @@
         <v>82</v>
       </c>
       <c r="B83" t="n">
-        <v>163.7452995841522</v>
+        <v>92.15961983013101</v>
       </c>
       <c r="C83" t="n">
-        <v>-1460.797498759141</v>
+        <v>-1465.007669860751</v>
       </c>
       <c r="D83" t="n">
-        <v>1624.542798343293</v>
+        <v>1557.167289690882</v>
       </c>
     </row>
     <row r="84">
@@ -1591,13 +1591,13 @@
         <v>83</v>
       </c>
       <c r="B84" t="n">
-        <v>165.631160515507</v>
+        <v>93.95425402431545</v>
       </c>
       <c r="C84" t="n">
-        <v>-1462.345451480338</v>
+        <v>-1466.697157961199</v>
       </c>
       <c r="D84" t="n">
-        <v>1627.976611995845</v>
+        <v>1560.651411985514</v>
       </c>
     </row>
     <row r="85">
@@ -1605,13 +1605,13 @@
         <v>84</v>
       </c>
       <c r="B85" t="n">
-        <v>168.3191875643343</v>
+        <v>101.8675310020882</v>
       </c>
       <c r="C85" t="n">
-        <v>-1463.038057058786</v>
+        <v>-1467.308591999444</v>
       </c>
       <c r="D85" t="n">
-        <v>1631.35724462312</v>
+        <v>1569.176123001532</v>
       </c>
     </row>
     <row r="86">
@@ -1619,13 +1619,13 @@
         <v>85</v>
       </c>
       <c r="B86" t="n">
-        <v>170.9901223873078</v>
+        <v>108.637780616982</v>
       </c>
       <c r="C86" t="n">
-        <v>-1467.559335407735</v>
+        <v>-1466.314313598209</v>
       </c>
       <c r="D86" t="n">
-        <v>1638.549457795044</v>
+        <v>1574.952094215191</v>
       </c>
     </row>
     <row r="87">
@@ -1633,13 +1633,13 @@
         <v>86</v>
       </c>
       <c r="B87" t="n">
-        <v>172.0587378718878</v>
+        <v>112.265619852081</v>
       </c>
       <c r="C87" t="n">
-        <v>-1470.592684676167</v>
+        <v>-1466.708792638137</v>
       </c>
       <c r="D87" t="n">
-        <v>1642.651422548055</v>
+        <v>1578.974412490218</v>
       </c>
     </row>
     <row r="88">
@@ -1647,13 +1647,13 @@
         <v>87</v>
       </c>
       <c r="B88" t="n">
-        <v>176.8176855438271</v>
+        <v>123.291480067591</v>
       </c>
       <c r="C88" t="n">
-        <v>-1476.960919529302</v>
+        <v>-1468.893564171144</v>
       </c>
       <c r="D88" t="n">
-        <v>1653.77860507313</v>
+        <v>1592.185044238736</v>
       </c>
     </row>
     <row r="89">
@@ -1661,13 +1661,13 @@
         <v>88</v>
       </c>
       <c r="B89" t="n">
-        <v>175.327961605554</v>
+        <v>122.3961143552247</v>
       </c>
       <c r="C89" t="n">
-        <v>-1481.252610073119</v>
+        <v>-1468.958483786924</v>
       </c>
       <c r="D89" t="n">
-        <v>1656.580571678673</v>
+        <v>1591.354598142148</v>
       </c>
     </row>
     <row r="90">
@@ -1675,13 +1675,13 @@
         <v>89</v>
       </c>
       <c r="B90" t="n">
-        <v>181.1510414046651</v>
+        <v>127.5885113237645</v>
       </c>
       <c r="C90" t="n">
-        <v>-1485.513123137456</v>
+        <v>-1473.459938554848</v>
       </c>
       <c r="D90" t="n">
-        <v>1666.664164542121</v>
+        <v>1601.048449878612</v>
       </c>
     </row>
     <row r="91">
@@ -1689,13 +1689,13 @@
         <v>90</v>
       </c>
       <c r="B91" t="n">
-        <v>183.7389160785465</v>
+        <v>133.2928146191868</v>
       </c>
       <c r="C91" t="n">
-        <v>-1487.579453863596</v>
+        <v>-1474.380450948344</v>
       </c>
       <c r="D91" t="n">
-        <v>1671.318369942142</v>
+        <v>1607.67326556753</v>
       </c>
     </row>
     <row r="92">
@@ -1703,13 +1703,13 @@
         <v>91</v>
       </c>
       <c r="B92" t="n">
-        <v>184.1080107366586</v>
+        <v>136.061664821663</v>
       </c>
       <c r="C92" t="n">
-        <v>-1495.002181505703</v>
+        <v>-1479.751052619013</v>
       </c>
       <c r="D92" t="n">
-        <v>1679.110192242362</v>
+        <v>1615.812717440676</v>
       </c>
     </row>
     <row r="93">
@@ -1717,13 +1717,13 @@
         <v>92</v>
       </c>
       <c r="B93" t="n">
-        <v>185.5269852081587</v>
+        <v>132.0312418610294</v>
       </c>
       <c r="C93" t="n">
-        <v>-1499.438993669405</v>
+        <v>-1484.897695740194</v>
       </c>
       <c r="D93" t="n">
-        <v>1684.965978877564</v>
+        <v>1616.928937601223</v>
       </c>
     </row>
     <row r="94">
@@ -1731,13 +1731,13 @@
         <v>93</v>
       </c>
       <c r="B94" t="n">
-        <v>180.3079946933085</v>
+        <v>151.5764128739878</v>
       </c>
       <c r="C94" t="n">
-        <v>-1512.143779892484</v>
+        <v>-1490.078755245495</v>
       </c>
       <c r="D94" t="n">
-        <v>1692.451774585793</v>
+        <v>1641.655168119483</v>
       </c>
     </row>
     <row r="95">
@@ -1745,13 +1745,13 @@
         <v>94</v>
       </c>
       <c r="B95" t="n">
-        <v>183.576775571026</v>
+        <v>137.3591762426661</v>
       </c>
       <c r="C95" t="n">
-        <v>-1511.827100038851</v>
+        <v>-1495.414004649008</v>
       </c>
       <c r="D95" t="n">
-        <v>1695.403875609877</v>
+        <v>1632.773180891674</v>
       </c>
     </row>
     <row r="96">
@@ -1759,13 +1759,13 @@
         <v>95</v>
       </c>
       <c r="B96" t="n">
-        <v>188.9333649159806</v>
+        <v>151.363693165634</v>
       </c>
       <c r="C96" t="n">
-        <v>-1512.965958334061</v>
+        <v>-1496.279487324296</v>
       </c>
       <c r="D96" t="n">
-        <v>1701.899323250042</v>
+        <v>1647.64318048993</v>
       </c>
     </row>
     <row r="97">
@@ -1773,13 +1773,13 @@
         <v>96</v>
       </c>
       <c r="B97" t="n">
-        <v>187.1878864816063</v>
+        <v>151.1046038667392</v>
       </c>
       <c r="C97" t="n">
-        <v>-1516.826958577898</v>
+        <v>-1495.631953614461</v>
       </c>
       <c r="D97" t="n">
-        <v>1704.014845059504</v>
+        <v>1646.7365574812</v>
       </c>
     </row>
     <row r="98">
@@ -1787,13 +1787,13 @@
         <v>97</v>
       </c>
       <c r="B98" t="n">
-        <v>186.3565262194426</v>
+        <v>155.2376778526387</v>
       </c>
       <c r="C98" t="n">
-        <v>-1519.669380086089</v>
+        <v>-1496.142603237382</v>
       </c>
       <c r="D98" t="n">
-        <v>1706.025906305532</v>
+        <v>1651.380281090021</v>
       </c>
     </row>
     <row r="99">
@@ -1801,13 +1801,13 @@
         <v>98</v>
       </c>
       <c r="B99" t="n">
-        <v>182.4450519695987</v>
+        <v>162.8422432658837</v>
       </c>
       <c r="C99" t="n">
-        <v>-1529.159414095721</v>
+        <v>-1497.460039414922</v>
       </c>
       <c r="D99" t="n">
-        <v>1711.60446606532</v>
+        <v>1660.302282680806</v>
       </c>
     </row>
     <row r="100">
@@ -1815,13 +1815,13 @@
         <v>99</v>
       </c>
       <c r="B100" t="n">
-        <v>167.8172655168001</v>
+        <v>189.5628530146679</v>
       </c>
       <c r="C100" t="n">
-        <v>-1541.8607700718</v>
+        <v>-1479.585541753225</v>
       </c>
       <c r="D100" t="n">
-        <v>1709.6780355886</v>
+        <v>1669.148394767893</v>
       </c>
     </row>
     <row r="101">
@@ -1829,13 +1829,13 @@
         <v>100</v>
       </c>
       <c r="B101" t="n">
-        <v>130.3924407958984</v>
+        <v>181.0143585205078</v>
       </c>
       <c r="C101" t="n">
-        <v>-1544.547470092773</v>
+        <v>-1442.149394989014</v>
       </c>
       <c r="D101" t="n">
-        <v>1674.939910888672</v>
+        <v>1623.163753509521</v>
       </c>
     </row>
   </sheetData>

</xml_diff>